<commit_message>
docs(roles): reflect 2026-04-25 admin limited-oversight tier
Permissions sheet:
- Manage add-on catalog: admin demoted ✅ → ❌ (CRUD now owner-only)
- Adjust add-on stock levels: admin demoted ✅ → ❌
- Deactivate / reactivate staff account: relabeled to "front-desk staff
  account" + admin granted ✅ (front_desk targets only — backend rejects
  other roles 403 and self 422)
- View activity log: admin granted ✅ (read-only — write paths stay
  system-only)
- Two new rows under "Limited oversight (admin tier)":
  - Toggle add-on enabled / disabled (catalog visibility only)
  - Toggle room status (available / renovation / maintenance / reserved /
    closed)

Rationale sheet: appended a new section explaining why these capabilities
pass the two-question test (no rate change, no staff structure change, no
compliance surface) but were previously bundled with strategic CRUD that
only owner needs.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roles.xlsx
+++ b/docs/roles.xlsx
@@ -88,7 +88,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -110,11 +110,55 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,6 +195,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -672,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -715,10 +761,10 @@
           <t>Self-service</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="15" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -915,10 +961,10 @@
           <t>Front-desk operations (counter work)</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="15" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1196,10 +1242,10 @@
           <t>Booking oversight (beyond today's shift)</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="15" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1342,10 +1388,10 @@
           <t>Guest communication</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="n"/>
+      <c r="E27" s="15" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -1488,10 +1534,10 @@
           <t>Content &amp; marketing</t>
         </is>
       </c>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
+      <c r="B33" s="14" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="15" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -1742,10 +1788,10 @@
           <t>Inventory (catalog, not strategic)</t>
         </is>
       </c>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="14" t="n"/>
+      <c r="E43" s="15" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -1765,7 +1811,7 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -1792,7 +1838,7 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
@@ -1834,10 +1880,10 @@
           <t>Strategic controls (owner-only)</t>
         </is>
       </c>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
+      <c r="E47" s="15" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -1980,10 +2026,10 @@
           <t>Staff management (owner-only)</t>
         </is>
       </c>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
+      <c r="E53" s="15" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
@@ -2042,7 +2088,7 @@
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Deactivate / reactivate staff account</t>
+          <t>Deactivate / reactivate a front-desk staff account</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
@@ -2057,7 +2103,7 @@
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
@@ -2099,10 +2145,10 @@
           <t>Analytics &amp; audit (owner-only)</t>
         </is>
       </c>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="14" t="n"/>
+      <c r="E58" s="15" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
@@ -2230,7 +2276,7 @@
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
@@ -2272,10 +2318,10 @@
           <t>Portal navigation</t>
         </is>
       </c>
-      <c r="B65" s="4" t="n"/>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="4" t="n"/>
-      <c r="E65" s="4" t="n"/>
+      <c r="B65" s="14" t="n"/>
+      <c r="C65" s="14" t="n"/>
+      <c r="D65" s="14" t="n"/>
+      <c r="E65" s="15" t="n"/>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
@@ -2455,10 +2501,76 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Limited oversight (admin tier — added 2026-04-25)</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="n"/>
+      <c r="C77" s="14" t="n"/>
+      <c r="D77" s="14" t="n"/>
+      <c r="E77" s="15" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Toggle add-on enabled / disabled (catalog visibility only)</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Toggle room status (available / renovation / maintenance / reserved / closed)</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A77:E77"/>
     <mergeCell ref="A65:E65"/>
     <mergeCell ref="A43:E43"/>
     <mergeCell ref="A2:E2"/>
@@ -2481,7 +2593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2613,6 +2725,34 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Limited oversight tier (added 2026-04-25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>On 2026-04-25 admin gained three narrow toggle endpoints on top of its existing day-to-day management scope: change a room's availability_status (available / renovation / maintenance / reserved / closed), toggle an addon's is_active, and toggle a front_desk user's is_active. These pass the two-question test (no rate change, no staff structure change, no compliance surface) but were previously bundled with strategic CRUD that only owner needs. Splitting them out lets admin enable/disable items in the catalog without granting create/rename/reprice/delete. Backend boundary lives in controller methods, not just middleware: toggleActive on users returns 422 on self-toggle and 403 on any non-front_desk target. Eight feature tests in SecurityAuditTest lock the matrix down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Same date: addons CRUD (POST/PATCH/DELETE) was demoted from admin_or_owner to admin_role (owner-only). Renaming or repricing an addon is structurally equivalent to changing inventory and pricing, so it sits with rooms CRUD on the owner side. The toggle stays admin-eligible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Activity log gained a read role for admin (write-only-by-system stays — admin doesn't author audit entries). Reading the log is a transparency capability, not a privilege escalation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>